<commit_message>
Updated GBR_grids_kan10 model - 2026-07-09 13:52
</commit_message>
<xml_diff>
--- a/VerveStacks_GBR_grids_kan10/Sets-vervestacks.xlsx
+++ b/VerveStacks_GBR_grids_kan10/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GBR_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2000C7E6-66D2-4752-AD67-808BDC2C9585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF324351-EFC1-42C4-A80C-3D6518EF466C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="295">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -364,115 +364,109 @@
     <t>t_pos_andor</t>
   </si>
   <si>
+    <t>p_w1262971878_GBR</t>
+  </si>
+  <si>
+    <t>e_w1262971878_GBR*</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>p_w1274396508-400_GBR</t>
+  </si>
+  <si>
+    <t>e_w1274396508-400_GBR*</t>
+  </si>
+  <si>
+    <t>p_w137050527_GBR</t>
+  </si>
+  <si>
+    <t>e_w137050527_GBR*</t>
+  </si>
+  <si>
+    <t>p_w148382435_GBR</t>
+  </si>
+  <si>
+    <t>e_w148382435_GBR*</t>
+  </si>
+  <si>
+    <t>p_w25422135-400_GBR</t>
+  </si>
+  <si>
+    <t>e_w25422135-400_GBR*</t>
+  </si>
+  <si>
+    <t>p_w297840585_GBR</t>
+  </si>
+  <si>
+    <t>e_w297840585_GBR*</t>
+  </si>
+  <si>
+    <t>p_w375626500_GBR</t>
+  </si>
+  <si>
+    <t>e_w375626500_GBR*</t>
+  </si>
+  <si>
+    <t>p_w568527671_GBR</t>
+  </si>
+  <si>
+    <t>e_w568527671_GBR*</t>
+  </si>
+  <si>
+    <t>p_w975637991_GBR</t>
+  </si>
+  <si>
+    <t>e_w975637991_GBR*</t>
+  </si>
+  <si>
     <t>p_r10695345_GBR</t>
   </si>
   <si>
     <t>e_r10695345_GBR*</t>
   </si>
   <si>
-    <t>OR</t>
-  </si>
-  <si>
     <t>p_w1078532568_GBR</t>
   </si>
   <si>
     <t>e_w1078532568_GBR*</t>
   </si>
   <si>
+    <t>p_w109189896_GBR</t>
+  </si>
+  <si>
+    <t>e_w109189896_GBR*</t>
+  </si>
+  <si>
     <t>p_w23281217_GBR</t>
   </si>
   <si>
     <t>e_w23281217_GBR*</t>
   </si>
   <si>
+    <t>p_w536905500_GBR</t>
+  </si>
+  <si>
+    <t>e_w536905500_GBR*</t>
+  </si>
+  <si>
     <t>p_w636630368_GBR</t>
   </si>
   <si>
     <t>e_w636630368_GBR*</t>
   </si>
   <si>
+    <t>p_w642490160_GBR</t>
+  </si>
+  <si>
+    <t>e_w642490160_GBR*</t>
+  </si>
+  <si>
     <t>p_w775577829_GBR</t>
   </si>
   <si>
     <t>e_w775577829_GBR*</t>
-  </si>
-  <si>
-    <t>p_w1262971878_GBR</t>
-  </si>
-  <si>
-    <t>e_w1262971878_GBR*</t>
-  </si>
-  <si>
-    <t>p_w1274396508-400_GBR</t>
-  </si>
-  <si>
-    <t>e_w1274396508-400_GBR*</t>
-  </si>
-  <si>
-    <t>p_w137050527_GBR</t>
-  </si>
-  <si>
-    <t>e_w137050527_GBR*</t>
-  </si>
-  <si>
-    <t>p_w148382435_GBR</t>
-  </si>
-  <si>
-    <t>e_w148382435_GBR*</t>
-  </si>
-  <si>
-    <t>p_w25422135-400_GBR</t>
-  </si>
-  <si>
-    <t>e_w25422135-400_GBR*</t>
-  </si>
-  <si>
-    <t>p_w297840585_GBR</t>
-  </si>
-  <si>
-    <t>e_w297840585_GBR*</t>
-  </si>
-  <si>
-    <t>p_w375626500_GBR</t>
-  </si>
-  <si>
-    <t>e_w375626500_GBR*</t>
-  </si>
-  <si>
-    <t>p_w568527671_GBR</t>
-  </si>
-  <si>
-    <t>e_w568527671_GBR*</t>
-  </si>
-  <si>
-    <t>p_w975637991_GBR</t>
-  </si>
-  <si>
-    <t>e_w975637991_GBR*</t>
-  </si>
-  <si>
-    <t>p_w109189896_GBR</t>
-  </si>
-  <si>
-    <t>e_w109189896_GBR*</t>
-  </si>
-  <si>
-    <t>p_w536905500_GBR</t>
-  </si>
-  <si>
-    <t>e_w536905500_GBR*</t>
-  </si>
-  <si>
-    <t>p_w642490160_GBR</t>
-  </si>
-  <si>
-    <t>e_w642490160_GBR*</t>
-  </si>
-  <si>
-    <t>p_w227767019-275_GBR</t>
-  </si>
-  <si>
-    <t>e_w227767019-275_GBR*</t>
   </si>
   <si>
     <t>rez_spv_GBR_001</t>
@@ -1773,8 +1767,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4A70EC-5A91-4C91-982D-8C5ACA6787A5}">
-  <dimension ref="B9:E104"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{771D7C22-59A4-461D-896E-A76CD60F2D3D}">
+  <dimension ref="B9:E103"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -3095,20 +3089,6 @@
         <v>294</v>
       </c>
       <c r="E103" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="104" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B104" t="s">
-        <v>295</v>
-      </c>
-      <c r="C104" t="s">
-        <v>296</v>
-      </c>
-      <c r="D104" t="s">
-        <v>296</v>
-      </c>
-      <c r="E104" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>